<commit_message>
actualización lat lon dir
</commit_message>
<xml_diff>
--- a/Data/Clean/base_final.xlsx
+++ b/Data/Clean/base_final.xlsx
@@ -1,26 +1,19 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
-  <workbookPr defaultThemeVersion="202300"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/4d57902ee1d42ba8/Documentos/GitHub/DoingEconomics_Proyect/Data/Clean/"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="25" documentId="11_305B94D7CC1AB73EA06E5FA5F4012D16618C957F" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C3BFC030-78AB-4F0F-A9D1-35555FF8F04C}"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <workbookPr/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView activeTab="0"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="1" r:id="rId2"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <calcPr calcId="125725" fullCalcOnLoad="true"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="851" uniqueCount="202">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" count="895" uniqueCount="246">
   <si>
     <t>Restaurante con encuesta aplicada (1=Si, 0=No)</t>
   </si>
@@ -626,39 +619,159 @@
   </si>
   <si>
     <t>Nº 70 de 640 hoteles en Bogotá</t>
+  </si>
+  <si>
+    <t>lat</t>
+  </si>
+  <si>
+    <t>lon</t>
+  </si>
+  <si>
+    <t>direccion</t>
+  </si>
+  <si>
+    <t>Cra. 12a #83 - 11, Vapiano, Bogotá, Colombia</t>
+  </si>
+  <si>
+    <t>Kr 13 #82-36, Bogotá, Colombia</t>
+  </si>
+  <si>
+    <t>Cra. 4a #27-54, Santa Fé, Bogotá, Cundinamarca, Colombia</t>
+  </si>
+  <si>
+    <t>Cra. 11a #93b-12, Bogotá, Colombia</t>
+  </si>
+  <si>
+    <t>Cl. 82 #12a - 35, Chapinero, Bogotá, Cundinamarca, Colombia</t>
+  </si>
+  <si>
+    <t>Cra. 24 #41-22, Bogotá, Colombia</t>
+  </si>
+  <si>
+    <t>Kr 13 #85-85, Bogotá, Colombia</t>
+  </si>
+  <si>
+    <t>salón 2, Calle 85 #12-66 Piso 15, Bogotá, Colombia</t>
+  </si>
+  <si>
+    <t>Cra. 12a #83-64, Bogotá, Colombia</t>
+  </si>
+  <si>
+    <t>Passage Santa Cruz de Mompox, Cl. 27 Bis #6-51 local 1, Santa Fé, Bogotá, Cundinamarca, Colombia</t>
+  </si>
+  <si>
+    <t>Cl. 119b #6a-18, Usaquén, Bogotá, Cundinamarca, Colombia</t>
+  </si>
+  <si>
+    <t>Cl. 65 #4a-51, Bogotá, Colombia</t>
+  </si>
+  <si>
+    <t>Kr 13 #85 - 24, Bogotá, Colombia</t>
+  </si>
+  <si>
+    <t>Cl. 26c #4a - 15, Bogotá, Colombia</t>
+  </si>
+  <si>
+    <t>Esquina Calle 95, Cra. 48, Bogotá, Colombia</t>
+  </si>
+  <si>
+    <t>Cra. 12a #83 - 30, Bogotá, Colombia</t>
+  </si>
+  <si>
+    <t>Cl. 79b #8-61, Bogotá, Colombia</t>
+  </si>
+  <si>
+    <t>Cl. 81 #13-05, Chapinero, Bogotá, Cundinamarca, Colombia</t>
+  </si>
+  <si>
+    <t>Av 19 con calle 100-52, Usaquén, Bogotá, Cundinamarca, Colombia</t>
+  </si>
+  <si>
+    <t>Ak 7 #120 #20, Usaquén, Bogotá, Cundinamarca, Colombia</t>
+  </si>
+  <si>
+    <t>Cl. 61 #5-30, Chapinero, Bogotá, Cundinamarca, Colombia</t>
+  </si>
+  <si>
+    <t>Cl. 69a #6-24, Chapinero, Bogotá, Cundinamarca, Colombia</t>
+  </si>
+  <si>
+    <t>Cl. 140 #13-62, Usaquén, Bogotá, Cundinamarca, Colombia</t>
+  </si>
+  <si>
+    <t>Cl. 93a #12-35, Chapinero, Bogotá, Cundinamarca, Colombia</t>
+  </si>
+  <si>
+    <t>Cl. 117 #6a-60, Usaquén, Bogotá, Cundinamarca, Colombia</t>
+  </si>
+  <si>
+    <t>Calle 43 # 19-18 Bogota, Teusaquillo, Bogotá, Cundinamarca, Colombia</t>
+  </si>
+  <si>
+    <t>Ak 7 #72-74, Bogotá, Colombia</t>
+  </si>
+  <si>
+    <t>Cl. 117 #6a-61, Usaquén, Bogotá, Cundinamarca, Colombia</t>
+  </si>
+  <si>
+    <t>Cra. 12 #97-04, Bogotá, Colombia</t>
+  </si>
+  <si>
+    <t>Ac 116 #15-71 2do piso, Bogotá, Colombia</t>
+  </si>
+  <si>
+    <t>Cra. 29b #72, Bogotá, Colombia</t>
+  </si>
+  <si>
+    <t>Cra. 4a #26C-23, Bogotá, Colombia</t>
+  </si>
+  <si>
+    <t>Cra. 6 #69a - 23, Rosales, Bogotá, Colombia</t>
+  </si>
+  <si>
+    <t>Cl. 93 #11-19, Bogotá, Colombia</t>
+  </si>
+  <si>
+    <t>OFICINA PRINCIPAL MONTENEGRO FACILISIMO, Cra. 5 #15-22, Santa Fé, MONTENEGRO, Bogotá, Quindío, Colombia</t>
+  </si>
+  <si>
+    <t>Cl. 75 #20c-89, Bogotá, Colombia</t>
+  </si>
+  <si>
+    <t>Cl. 68 #6 - 39, Bogotá, Colombia</t>
+  </si>
+  <si>
+    <t>Cl. 12b #0-57, La Candelaria, Bogotá, Colombia</t>
+  </si>
+  <si>
+    <t>Cl. 73 #9-42, Bogotá, Colombia</t>
+  </si>
+  <si>
+    <t>Ac 100 #1973 a 19a-97, Bogotá, Colombia</t>
+  </si>
+  <si>
+    <t>Ac 116 #53 - 26, Bogotá, Colombia</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <fonts count="1">
     <font>
       <sz val="11"/>
       <name val="Calibri"/>
     </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-    </font>
   </fonts>
-  <fills count="3">
+  <fills count="2">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFC000"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
   </fills>
-  <borders count="6">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -666,559 +779,131 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="medium">
-        <color indexed="64"/>
-      </left>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top style="medium">
-        <color indexed="64"/>
-      </top>
-      <bottom style="medium">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top style="medium">
-        <color indexed="64"/>
-      </top>
-      <bottom style="medium">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right/>
-      <top style="medium">
-        <color indexed="64"/>
-      </top>
-      <bottom style="medium">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right style="medium">
-        <color indexed="64"/>
-      </right>
-      <top style="medium">
-        <color indexed="64"/>
-      </top>
-      <bottom style="medium">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
+    <border/>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="1" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="true"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="0"/>
-  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
-    </ext>
-  </extLst>
 </styleSheet>
 </file>
 
-<file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
-  <a:themeElements>
-    <a:clrScheme name="Office">
-      <a:dk1>
-        <a:sysClr val="windowText" lastClr="000000"/>
-      </a:dk1>
-      <a:lt1>
-        <a:sysClr val="window" lastClr="FFFFFF"/>
-      </a:lt1>
-      <a:dk2>
-        <a:srgbClr val="0E2841"/>
-      </a:dk2>
-      <a:lt2>
-        <a:srgbClr val="E8E8E8"/>
-      </a:lt2>
-      <a:accent1>
-        <a:srgbClr val="156082"/>
-      </a:accent1>
-      <a:accent2>
-        <a:srgbClr val="E97132"/>
-      </a:accent2>
-      <a:accent3>
-        <a:srgbClr val="196B24"/>
-      </a:accent3>
-      <a:accent4>
-        <a:srgbClr val="0F9ED5"/>
-      </a:accent4>
-      <a:accent5>
-        <a:srgbClr val="A02B93"/>
-      </a:accent5>
-      <a:accent6>
-        <a:srgbClr val="4EA72E"/>
-      </a:accent6>
-      <a:hlink>
-        <a:srgbClr val="467886"/>
-      </a:hlink>
-      <a:folHlink>
-        <a:srgbClr val="96607D"/>
-      </a:folHlink>
-    </a:clrScheme>
-    <a:fontScheme name="Office">
-      <a:majorFont>
-        <a:latin typeface="Aptos Display" panose="02110004020202020204"/>
-        <a:ea typeface=""/>
-        <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="游ゴシック Light"/>
-        <a:font script="Hang" typeface="맑은 고딕"/>
-        <a:font script="Hans" typeface="等线 Light"/>
-        <a:font script="Hant" typeface="新細明體"/>
-        <a:font script="Arab" typeface="Times New Roman"/>
-        <a:font script="Hebr" typeface="Times New Roman"/>
-        <a:font script="Thai" typeface="Tahoma"/>
-        <a:font script="Ethi" typeface="Nyala"/>
-        <a:font script="Beng" typeface="Vrinda"/>
-        <a:font script="Gujr" typeface="Shruti"/>
-        <a:font script="Khmr" typeface="MoolBoran"/>
-        <a:font script="Knda" typeface="Tunga"/>
-        <a:font script="Guru" typeface="Raavi"/>
-        <a:font script="Cans" typeface="Euphemia"/>
-        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
-        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
-        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
-        <a:font script="Thaa" typeface="MV Boli"/>
-        <a:font script="Deva" typeface="Mangal"/>
-        <a:font script="Telu" typeface="Gautami"/>
-        <a:font script="Taml" typeface="Latha"/>
-        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
-        <a:font script="Orya" typeface="Kalinga"/>
-        <a:font script="Mlym" typeface="Kartika"/>
-        <a:font script="Laoo" typeface="DokChampa"/>
-        <a:font script="Sinh" typeface="Iskoola Pota"/>
-        <a:font script="Mong" typeface="Mongolian Baiti"/>
-        <a:font script="Viet" typeface="Times New Roman"/>
-        <a:font script="Uigh" typeface="Microsoft Uighur"/>
-        <a:font script="Geor" typeface="Sylfaen"/>
-        <a:font script="Armn" typeface="Arial"/>
-        <a:font script="Bugi" typeface="Leelawadee UI"/>
-        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
-        <a:font script="Java" typeface="Javanese Text"/>
-        <a:font script="Lisu" typeface="Segoe UI"/>
-        <a:font script="Mymr" typeface="Myanmar Text"/>
-        <a:font script="Nkoo" typeface="Ebrima"/>
-        <a:font script="Olck" typeface="Nirmala UI"/>
-        <a:font script="Osma" typeface="Ebrima"/>
-        <a:font script="Phag" typeface="Phagspa"/>
-        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
-        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
-        <a:font script="Syre" typeface="Estrangelo Edessa"/>
-        <a:font script="Sora" typeface="Nirmala UI"/>
-        <a:font script="Tale" typeface="Microsoft Tai Le"/>
-        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
-        <a:font script="Tfng" typeface="Ebrima"/>
-      </a:majorFont>
-      <a:minorFont>
-        <a:latin typeface="Aptos Narrow" panose="02110004020202020204"/>
-        <a:ea typeface=""/>
-        <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="游ゴシック"/>
-        <a:font script="Hang" typeface="맑은 고딕"/>
-        <a:font script="Hans" typeface="等线"/>
-        <a:font script="Hant" typeface="新細明體"/>
-        <a:font script="Arab" typeface="Arial"/>
-        <a:font script="Hebr" typeface="Arial"/>
-        <a:font script="Thai" typeface="Tahoma"/>
-        <a:font script="Ethi" typeface="Nyala"/>
-        <a:font script="Beng" typeface="Vrinda"/>
-        <a:font script="Gujr" typeface="Shruti"/>
-        <a:font script="Khmr" typeface="DaunPenh"/>
-        <a:font script="Knda" typeface="Tunga"/>
-        <a:font script="Guru" typeface="Raavi"/>
-        <a:font script="Cans" typeface="Euphemia"/>
-        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
-        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
-        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
-        <a:font script="Thaa" typeface="MV Boli"/>
-        <a:font script="Deva" typeface="Mangal"/>
-        <a:font script="Telu" typeface="Gautami"/>
-        <a:font script="Taml" typeface="Latha"/>
-        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
-        <a:font script="Orya" typeface="Kalinga"/>
-        <a:font script="Mlym" typeface="Kartika"/>
-        <a:font script="Laoo" typeface="DokChampa"/>
-        <a:font script="Sinh" typeface="Iskoola Pota"/>
-        <a:font script="Mong" typeface="Mongolian Baiti"/>
-        <a:font script="Viet" typeface="Arial"/>
-        <a:font script="Uigh" typeface="Microsoft Uighur"/>
-        <a:font script="Geor" typeface="Sylfaen"/>
-        <a:font script="Armn" typeface="Arial"/>
-        <a:font script="Bugi" typeface="Leelawadee UI"/>
-        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
-        <a:font script="Java" typeface="Javanese Text"/>
-        <a:font script="Lisu" typeface="Segoe UI"/>
-        <a:font script="Mymr" typeface="Myanmar Text"/>
-        <a:font script="Nkoo" typeface="Ebrima"/>
-        <a:font script="Olck" typeface="Nirmala UI"/>
-        <a:font script="Osma" typeface="Ebrima"/>
-        <a:font script="Phag" typeface="Phagspa"/>
-        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
-        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
-        <a:font script="Syre" typeface="Estrangelo Edessa"/>
-        <a:font script="Sora" typeface="Nirmala UI"/>
-        <a:font script="Tale" typeface="Microsoft Tai Le"/>
-        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
-        <a:font script="Tfng" typeface="Ebrima"/>
-      </a:minorFont>
-    </a:fontScheme>
-    <a:fmtScheme name="Office">
-      <a:fillStyleLst>
-        <a:solidFill>
-          <a:schemeClr val="phClr"/>
-        </a:solidFill>
-        <a:gradFill rotWithShape="1">
-          <a:gsLst>
-            <a:gs pos="0">
-              <a:schemeClr val="phClr">
-                <a:lumMod val="110000"/>
-                <a:satMod val="105000"/>
-                <a:tint val="67000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="50000">
-              <a:schemeClr val="phClr">
-                <a:lumMod val="105000"/>
-                <a:satMod val="103000"/>
-                <a:tint val="73000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="100000">
-              <a:schemeClr val="phClr">
-                <a:lumMod val="105000"/>
-                <a:satMod val="109000"/>
-                <a:tint val="81000"/>
-              </a:schemeClr>
-            </a:gs>
-          </a:gsLst>
-          <a:lin ang="5400000" scaled="0"/>
-        </a:gradFill>
-        <a:gradFill rotWithShape="1">
-          <a:gsLst>
-            <a:gs pos="0">
-              <a:schemeClr val="phClr">
-                <a:satMod val="103000"/>
-                <a:lumMod val="102000"/>
-                <a:tint val="94000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="50000">
-              <a:schemeClr val="phClr">
-                <a:satMod val="110000"/>
-                <a:lumMod val="100000"/>
-                <a:shade val="100000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="100000">
-              <a:schemeClr val="phClr">
-                <a:lumMod val="99000"/>
-                <a:satMod val="120000"/>
-                <a:shade val="78000"/>
-              </a:schemeClr>
-            </a:gs>
-          </a:gsLst>
-          <a:lin ang="5400000" scaled="0"/>
-        </a:gradFill>
-      </a:fillStyleLst>
-      <a:lnStyleLst>
-        <a:ln w="12700" cap="flat" cmpd="sng" algn="ctr">
-          <a:solidFill>
-            <a:schemeClr val="phClr"/>
-          </a:solidFill>
-          <a:prstDash val="solid"/>
-          <a:miter lim="800000"/>
-        </a:ln>
-        <a:ln w="19050" cap="flat" cmpd="sng" algn="ctr">
-          <a:solidFill>
-            <a:schemeClr val="phClr"/>
-          </a:solidFill>
-          <a:prstDash val="solid"/>
-          <a:miter lim="800000"/>
-        </a:ln>
-        <a:ln w="25400" cap="flat" cmpd="sng" algn="ctr">
-          <a:solidFill>
-            <a:schemeClr val="phClr"/>
-          </a:solidFill>
-          <a:prstDash val="solid"/>
-          <a:miter lim="800000"/>
-        </a:ln>
-      </a:lnStyleLst>
-      <a:effectStyleLst>
-        <a:effectStyle>
-          <a:effectLst/>
-        </a:effectStyle>
-        <a:effectStyle>
-          <a:effectLst/>
-        </a:effectStyle>
-        <a:effectStyle>
-          <a:effectLst>
-            <a:outerShdw blurRad="57150" dist="19050" dir="5400000" algn="ctr" rotWithShape="0">
-              <a:srgbClr val="000000">
-                <a:alpha val="63000"/>
-              </a:srgbClr>
-            </a:outerShdw>
-          </a:effectLst>
-        </a:effectStyle>
-      </a:effectStyleLst>
-      <a:bgFillStyleLst>
-        <a:solidFill>
-          <a:schemeClr val="phClr"/>
-        </a:solidFill>
-        <a:solidFill>
-          <a:schemeClr val="phClr">
-            <a:tint val="95000"/>
-            <a:satMod val="170000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:gradFill rotWithShape="1">
-          <a:gsLst>
-            <a:gs pos="0">
-              <a:schemeClr val="phClr">
-                <a:tint val="93000"/>
-                <a:satMod val="150000"/>
-                <a:shade val="98000"/>
-                <a:lumMod val="102000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="50000">
-              <a:schemeClr val="phClr">
-                <a:tint val="98000"/>
-                <a:satMod val="130000"/>
-                <a:shade val="90000"/>
-                <a:lumMod val="103000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="100000">
-              <a:schemeClr val="phClr">
-                <a:shade val="63000"/>
-                <a:satMod val="120000"/>
-              </a:schemeClr>
-            </a:gs>
-          </a:gsLst>
-          <a:lin ang="5400000" scaled="0"/>
-        </a:gradFill>
-      </a:bgFillStyleLst>
-    </a:fmtScheme>
-  </a:themeElements>
-  <a:objectDefaults>
-    <a:lnDef>
-      <a:spPr/>
-      <a:bodyPr/>
-      <a:lstStyle/>
-      <a:style>
-        <a:lnRef idx="2">
-          <a:schemeClr val="accent1"/>
-        </a:lnRef>
-        <a:fillRef idx="0">
-          <a:schemeClr val="accent1"/>
-        </a:fillRef>
-        <a:effectRef idx="1">
-          <a:schemeClr val="accent1"/>
-        </a:effectRef>
-        <a:fontRef idx="minor">
-          <a:schemeClr val="tx1"/>
-        </a:fontRef>
-      </a:style>
-    </a:lnDef>
-  </a:objectDefaults>
-  <a:extraClrSchemeLst/>
-  <a:extLst>
-    <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{2E142A2C-CD16-42D6-873A-C26D2A0506FA}" vid="{1BDDFF52-6CD6-40A5-AB3C-68EB2F1E4D0A}"/>
-    </a:ext>
-  </a:extLst>
-</a:theme>
-</file>
-
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:AE42"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
-  <cols>
-    <col min="1" max="1" width="11.21875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="54.88671875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="19.44140625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="39.109375" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="11.77734375" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="13" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="10.6640625" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="45" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="45.21875" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="27.6640625" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="175.5546875" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="86.21875" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="40.44140625" bestFit="1" customWidth="1"/>
-    <col min="15" max="17" width="13.44140625" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="22.6640625" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="39.5546875" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="32.6640625" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="35.44140625" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="37.6640625" bestFit="1" customWidth="1"/>
-    <col min="23" max="23" width="109.5546875" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="41.77734375" bestFit="1" customWidth="1"/>
-    <col min="25" max="25" width="49" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="10.21875" bestFit="1" customWidth="1"/>
-    <col min="27" max="27" width="12.33203125" bestFit="1" customWidth="1"/>
-    <col min="28" max="28" width="11.21875" bestFit="1" customWidth="1"/>
-    <col min="29" max="29" width="10.6640625" bestFit="1" customWidth="1"/>
-    <col min="30" max="30" width="12.109375" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="41.6640625" style="8" bestFit="1" customWidth="1"/>
-    <col min="32" max="16384" width="8.88671875" style="5"/>
-  </cols>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:AH42"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:31" s="6" customFormat="1" ht="43.2" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="3" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="3" t="s">
+    <row r="1">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="3" t="s">
+      <c r="D1" t="s">
         <v>44</v>
       </c>
-      <c r="E1" s="3" t="s">
+      <c r="E1" t="s">
         <v>62</v>
       </c>
-      <c r="F1" s="3" t="s">
+      <c r="F1" t="s">
         <v>67</v>
       </c>
-      <c r="G1" s="3" t="s">
+      <c r="G1" t="s">
         <v>70</v>
       </c>
-      <c r="H1" s="3" t="s">
+      <c r="H1" t="s">
         <v>71</v>
       </c>
-      <c r="I1" s="3" t="s">
+      <c r="I1" t="s">
         <v>72</v>
       </c>
-      <c r="J1" s="3" t="s">
+      <c r="J1" t="s">
         <v>78</v>
       </c>
-      <c r="K1" s="3" t="s">
+      <c r="K1" t="s">
         <v>83</v>
       </c>
-      <c r="L1" s="3" t="s">
+      <c r="L1" t="s">
         <v>89</v>
       </c>
-      <c r="M1" s="3" t="s">
+      <c r="M1" t="s">
         <v>98</v>
       </c>
-      <c r="N1" s="3" t="s">
+      <c r="N1" t="s">
         <v>107</v>
       </c>
-      <c r="O1" s="3" t="s">
+      <c r="O1" t="s">
         <v>114</v>
       </c>
-      <c r="P1" s="3" t="s">
+      <c r="P1" t="s">
         <v>115</v>
       </c>
-      <c r="Q1" s="3" t="s">
+      <c r="Q1" t="s">
         <v>116</v>
       </c>
-      <c r="R1" s="3" t="s">
+      <c r="R1" t="s">
         <v>117</v>
       </c>
-      <c r="S1" s="3" t="s">
+      <c r="S1" t="s">
         <v>121</v>
       </c>
-      <c r="T1" s="3" t="s">
+      <c r="T1" t="s">
         <v>126</v>
       </c>
-      <c r="U1" s="3" t="s">
+      <c r="U1" t="s">
         <v>131</v>
       </c>
-      <c r="V1" s="3" t="s">
+      <c r="V1" t="s">
         <v>135</v>
       </c>
-      <c r="W1" s="3" t="s">
+      <c r="W1" t="s">
         <v>140</v>
       </c>
-      <c r="X1" s="3" t="s">
+      <c r="X1" t="s">
         <v>153</v>
       </c>
-      <c r="Y1" s="3" t="s">
+      <c r="Y1" t="s">
         <v>159</v>
       </c>
-      <c r="Z1" s="3" t="s">
+      <c r="Z1" t="s">
         <v>164</v>
       </c>
-      <c r="AA1" s="3" t="s">
+      <c r="AA1" t="s">
         <v>165</v>
       </c>
-      <c r="AB1" s="3" t="s">
+      <c r="AB1" t="s">
         <v>166</v>
       </c>
-      <c r="AC1" s="3" t="s">
+      <c r="AC1" t="s">
         <v>167</v>
       </c>
-      <c r="AD1" s="4" t="s">
+      <c r="AD1" t="s">
         <v>168</v>
       </c>
-      <c r="AE1" s="7" t="s">
+      <c r="AE1" t="s">
         <v>169</v>
       </c>
+      <c r="AF1" t="s">
+        <v>202</v>
+      </c>
+      <c r="AG1" t="s">
+        <v>203</v>
+      </c>
+      <c r="AH1" t="s">
+        <v>204</v>
+      </c>
     </row>
-    <row r="2" spans="1:31" x14ac:dyDescent="0.3">
+    <row r="2">
       <c r="A2" s="1">
         <v>1</v>
       </c>
@@ -1298,7 +983,7 @@
         <v>10053</v>
       </c>
       <c r="AA2" s="1">
-        <v>4.7</v>
+        <v>4.7000000000000002</v>
       </c>
       <c r="AB2" s="1">
         <v>1</v>
@@ -1307,13 +992,22 @@
         <v>190</v>
       </c>
       <c r="AD2" s="1">
-        <v>3.7</v>
-      </c>
-      <c r="AE2" s="8" t="s">
+        <v>3.7000000000000002</v>
+      </c>
+      <c r="AE2" t="s">
         <v>170</v>
       </c>
+      <c r="AF2" s="1">
+        <v>4.6676060000000001</v>
+      </c>
+      <c r="AG2" s="1">
+        <v>-74.054133999999991</v>
+      </c>
+      <c r="AH2" t="s">
+        <v>205</v>
+      </c>
     </row>
-    <row r="3" spans="1:31" x14ac:dyDescent="0.3">
+    <row r="3">
       <c r="A3" s="1">
         <v>1</v>
       </c>
@@ -1393,7 +1087,7 @@
         <v>7987</v>
       </c>
       <c r="AA3" s="1">
-        <v>4.7</v>
+        <v>4.7000000000000002</v>
       </c>
       <c r="AB3" s="1">
         <v>1</v>
@@ -1404,11 +1098,20 @@
       <c r="AD3" s="1">
         <v>4.9000000000000004</v>
       </c>
-      <c r="AE3" s="8" t="s">
+      <c r="AE3" t="s">
         <v>171</v>
       </c>
+      <c r="AF3" s="1">
+        <v>4.6672186999999994</v>
+      </c>
+      <c r="AG3" s="1">
+        <v>-74.054656800000004</v>
+      </c>
+      <c r="AH3" t="s">
+        <v>206</v>
+      </c>
     </row>
-    <row r="4" spans="1:31" x14ac:dyDescent="0.3">
+    <row r="4">
       <c r="A4" s="1">
         <v>1</v>
       </c>
@@ -1497,13 +1200,22 @@
         <v>231</v>
       </c>
       <c r="AD4" s="1">
-        <v>3.9</v>
-      </c>
-      <c r="AE4" s="8" t="s">
+        <v>3.8999999999999999</v>
+      </c>
+      <c r="AE4" t="s">
         <v>172</v>
       </c>
+      <c r="AF4" s="1">
+        <v>4.6143874999999994</v>
+      </c>
+      <c r="AG4" s="1">
+        <v>-74.066146599999996</v>
+      </c>
+      <c r="AH4" t="s">
+        <v>207</v>
+      </c>
     </row>
-    <row r="5" spans="1:31" x14ac:dyDescent="0.3">
+    <row r="5">
       <c r="A5" s="1">
         <v>1</v>
       </c>
@@ -1592,13 +1304,22 @@
         <v>825</v>
       </c>
       <c r="AD5" s="1">
-        <v>4.3</v>
-      </c>
-      <c r="AE5" s="8" t="s">
+        <v>4.2999999999999998</v>
+      </c>
+      <c r="AE5" t="s">
         <v>173</v>
       </c>
+      <c r="AF5" s="1">
+        <v>4.6768090999999998</v>
+      </c>
+      <c r="AG5" s="1">
+        <v>-74.047285700000003</v>
+      </c>
+      <c r="AH5" t="s">
+        <v>208</v>
+      </c>
     </row>
-    <row r="6" spans="1:31" x14ac:dyDescent="0.3">
+    <row r="6">
       <c r="A6" s="1">
         <v>0</v>
       </c>
@@ -1670,7 +1391,7 @@
         <v>2483</v>
       </c>
       <c r="AA6" s="1">
-        <v>4.8</v>
+        <v>4.7999999999999998</v>
       </c>
       <c r="AB6" s="1">
         <v>1</v>
@@ -1681,11 +1402,20 @@
       <c r="AD6" s="1">
         <v>4.5</v>
       </c>
-      <c r="AE6" s="8" t="s">
+      <c r="AE6" t="s">
         <v>174</v>
       </c>
+      <c r="AF6" s="1">
+        <v>4.6683975000000002</v>
+      </c>
+      <c r="AG6" s="1">
+        <v>-74.053802399999995</v>
+      </c>
+      <c r="AH6" t="s">
+        <v>209</v>
+      </c>
     </row>
-    <row r="7" spans="1:31" x14ac:dyDescent="0.3">
+    <row r="7">
       <c r="A7" s="1">
         <v>0</v>
       </c>
@@ -1768,11 +1498,20 @@
       <c r="AD7" s="1">
         <v>4.5</v>
       </c>
-      <c r="AE7" s="8" t="s">
+      <c r="AE7" t="s">
         <v>175</v>
       </c>
+      <c r="AF7" s="1">
+        <v>4.6317538999999996</v>
+      </c>
+      <c r="AG7" s="1">
+        <v>-74.074739199999996</v>
+      </c>
+      <c r="AH7" t="s">
+        <v>210</v>
+      </c>
     </row>
-    <row r="8" spans="1:31" x14ac:dyDescent="0.3">
+    <row r="8">
       <c r="A8" s="1">
         <v>1</v>
       </c>
@@ -1861,13 +1600,22 @@
         <v>529</v>
       </c>
       <c r="AD8" s="1">
-        <v>4.3</v>
-      </c>
-      <c r="AE8" s="8" t="s">
+        <v>4.2999999999999998</v>
+      </c>
+      <c r="AE8" t="s">
         <v>176</v>
       </c>
+      <c r="AF8" s="1">
+        <v>4.6702380000000003</v>
+      </c>
+      <c r="AG8" s="1">
+        <v>-74.053262000000004</v>
+      </c>
+      <c r="AH8" t="s">
+        <v>211</v>
+      </c>
     </row>
-    <row r="9" spans="1:31" x14ac:dyDescent="0.3">
+    <row r="9">
       <c r="A9" s="1">
         <v>1</v>
       </c>
@@ -1956,13 +1704,22 @@
         <v>114</v>
       </c>
       <c r="AD9" s="1">
-        <v>3.9</v>
-      </c>
-      <c r="AE9" s="8" t="s">
+        <v>3.8999999999999999</v>
+      </c>
+      <c r="AE9" t="s">
         <v>177</v>
       </c>
+      <c r="AF9" s="1">
+        <v>4.6690924999999996</v>
+      </c>
+      <c r="AG9" s="1">
+        <v>-74.053077899999991</v>
+      </c>
+      <c r="AH9" t="s">
+        <v>212</v>
+      </c>
     </row>
-    <row r="10" spans="1:31" x14ac:dyDescent="0.3">
+    <row r="10">
       <c r="A10" s="1">
         <v>0</v>
       </c>
@@ -2043,11 +1800,20 @@
         <v>0</v>
       </c>
       <c r="AD10" s="1"/>
-      <c r="AE10" s="8" t="s">
-        <v>48</v>
+      <c r="AE10" t="s">
+        <v>48</v>
+      </c>
+      <c r="AF10" s="1">
+        <v>4.6679246000000001</v>
+      </c>
+      <c r="AG10" s="1">
+        <v>-74.053489599999992</v>
+      </c>
+      <c r="AH10" t="s">
+        <v>213</v>
       </c>
     </row>
-    <row r="11" spans="1:31" x14ac:dyDescent="0.3">
+    <row r="11">
       <c r="A11" s="1">
         <v>1</v>
       </c>
@@ -2136,13 +1902,22 @@
         <v>419</v>
       </c>
       <c r="AD11" s="1">
-        <v>4.3</v>
-      </c>
-      <c r="AE11" s="8" t="s">
+        <v>4.2999999999999998</v>
+      </c>
+      <c r="AE11" t="s">
         <v>178</v>
       </c>
+      <c r="AF11" s="1">
+        <v>4.6144970000000001</v>
+      </c>
+      <c r="AG11" s="1">
+        <v>-74.068920199999994</v>
+      </c>
+      <c r="AH11" t="s">
+        <v>214</v>
+      </c>
     </row>
-    <row r="12" spans="1:31" x14ac:dyDescent="0.3">
+    <row r="12">
       <c r="A12" s="1">
         <v>1</v>
       </c>
@@ -2231,13 +2006,22 @@
         <v>16</v>
       </c>
       <c r="AD12" s="1">
-        <v>3.9</v>
-      </c>
-      <c r="AE12" s="8" t="s">
+        <v>3.8999999999999999</v>
+      </c>
+      <c r="AE12" t="s">
         <v>179</v>
       </c>
+      <c r="AF12" s="1">
+        <v>4.6963597000000004</v>
+      </c>
+      <c r="AG12" s="1">
+        <v>-74.030839300000011</v>
+      </c>
+      <c r="AH12" t="s">
+        <v>215</v>
+      </c>
     </row>
-    <row r="13" spans="1:31" x14ac:dyDescent="0.3">
+    <row r="13">
       <c r="A13" s="1">
         <v>1</v>
       </c>
@@ -2328,11 +2112,20 @@
       <c r="AD13" s="1">
         <v>4</v>
       </c>
-      <c r="AE13" s="8" t="s">
+      <c r="AE13" t="s">
         <v>180</v>
       </c>
+      <c r="AF13" s="1">
+        <v>4.6481026999999999</v>
+      </c>
+      <c r="AG13" s="1">
+        <v>-74.057687899999991</v>
+      </c>
+      <c r="AH13" t="s">
+        <v>216</v>
+      </c>
     </row>
-    <row r="14" spans="1:31" x14ac:dyDescent="0.3">
+    <row r="14">
       <c r="A14" s="1">
         <v>1</v>
       </c>
@@ -2421,13 +2214,22 @@
         <v>253</v>
       </c>
       <c r="AD14" s="1">
-        <v>4.3</v>
-      </c>
-      <c r="AE14" s="8" t="s">
+        <v>4.2999999999999998</v>
+      </c>
+      <c r="AE14" t="s">
         <v>181</v>
       </c>
+      <c r="AF14" s="1">
+        <v>4.6693340000000001</v>
+      </c>
+      <c r="AG14" s="1">
+        <v>-74.053410999999997</v>
+      </c>
+      <c r="AH14" t="s">
+        <v>217</v>
+      </c>
     </row>
-    <row r="15" spans="1:31" x14ac:dyDescent="0.3">
+    <row r="15">
       <c r="A15" s="1">
         <v>1</v>
       </c>
@@ -2518,11 +2320,20 @@
       <c r="AD15" s="1">
         <v>4.5</v>
       </c>
-      <c r="AE15" s="8" t="s">
+      <c r="AE15" t="s">
         <v>182</v>
       </c>
+      <c r="AF15" s="1">
+        <v>4.6127433</v>
+      </c>
+      <c r="AG15" s="1">
+        <v>-74.066767900000002</v>
+      </c>
+      <c r="AH15" t="s">
+        <v>218</v>
+      </c>
     </row>
-    <row r="16" spans="1:31" x14ac:dyDescent="0.3">
+    <row r="16">
       <c r="A16" s="1">
         <v>1</v>
       </c>
@@ -2602,7 +2413,7 @@
         <v>1117</v>
       </c>
       <c r="AA16" s="1">
-        <v>4.7</v>
+        <v>4.7000000000000002</v>
       </c>
       <c r="AB16" s="1">
         <v>1</v>
@@ -2613,11 +2424,20 @@
       <c r="AD16" s="1">
         <v>4</v>
       </c>
-      <c r="AE16" s="8" t="s">
+      <c r="AE16" t="s">
         <v>183</v>
       </c>
+      <c r="AF16" s="1">
+        <v>4.6833840000000002</v>
+      </c>
+      <c r="AG16" s="1">
+        <v>-74.060512199999991</v>
+      </c>
+      <c r="AH16" t="s">
+        <v>219</v>
+      </c>
     </row>
-    <row r="17" spans="1:31" x14ac:dyDescent="0.3">
+    <row r="17">
       <c r="A17" s="1">
         <v>1</v>
       </c>
@@ -2708,11 +2528,20 @@
       <c r="AD17" s="1">
         <v>4.5</v>
       </c>
-      <c r="AE17" s="8" t="s">
+      <c r="AE17" t="s">
         <v>184</v>
       </c>
+      <c r="AF17" s="1">
+        <v>4.6676150999999999</v>
+      </c>
+      <c r="AG17" s="1">
+        <v>-74.053812199999996</v>
+      </c>
+      <c r="AH17" t="s">
+        <v>220</v>
+      </c>
     </row>
-    <row r="18" spans="1:31" x14ac:dyDescent="0.3">
+    <row r="18">
       <c r="A18" s="1">
         <v>0</v>
       </c>
@@ -2795,11 +2624,20 @@
       <c r="AD18" s="1">
         <v>4.0999999999999996</v>
       </c>
-      <c r="AE18" s="8" t="s">
+      <c r="AE18" t="s">
         <v>185</v>
       </c>
+      <c r="AF18" s="1">
+        <v>4.6625094999999996</v>
+      </c>
+      <c r="AG18" s="1">
+        <v>-74.052126999999999</v>
+      </c>
+      <c r="AH18" t="s">
+        <v>221</v>
+      </c>
     </row>
-    <row r="19" spans="1:31" x14ac:dyDescent="0.3">
+    <row r="19">
       <c r="A19" s="1">
         <v>1</v>
       </c>
@@ -2890,11 +2728,20 @@
       <c r="AD19" s="1">
         <v>4.9000000000000004</v>
       </c>
-      <c r="AE19" s="8" t="s">
+      <c r="AE19" t="s">
         <v>186</v>
       </c>
+      <c r="AF19" s="1">
+        <v>4.6661218999999994</v>
+      </c>
+      <c r="AG19" s="1">
+        <v>-74.055825599999991</v>
+      </c>
+      <c r="AH19" t="s">
+        <v>222</v>
+      </c>
     </row>
-    <row r="20" spans="1:31" x14ac:dyDescent="0.3">
+    <row r="20">
       <c r="A20" s="1">
         <v>1</v>
       </c>
@@ -2985,11 +2832,20 @@
       <c r="AD20" s="1">
         <v>4.5</v>
       </c>
-      <c r="AE20" s="8" t="s">
+      <c r="AE20" t="s">
         <v>187</v>
       </c>
+      <c r="AF20" s="1">
+        <v>4.6868488000000008</v>
+      </c>
+      <c r="AG20" s="1">
+        <v>-74.051691300000002</v>
+      </c>
+      <c r="AH20" t="s">
+        <v>223</v>
+      </c>
     </row>
-    <row r="21" spans="1:31" x14ac:dyDescent="0.3">
+    <row r="21">
       <c r="A21" s="1">
         <v>1</v>
       </c>
@@ -3078,13 +2934,22 @@
         <v>220</v>
       </c>
       <c r="AD21" s="1">
-        <v>4.7</v>
-      </c>
-      <c r="AE21" s="8" t="s">
+        <v>4.7000000000000002</v>
+      </c>
+      <c r="AE21" t="s">
         <v>188</v>
       </c>
+      <c r="AF21" s="1">
+        <v>4.6967935000000001</v>
+      </c>
+      <c r="AG21" s="1">
+        <v>-74.030623399999996</v>
+      </c>
+      <c r="AH21" t="s">
+        <v>224</v>
+      </c>
     </row>
-    <row r="22" spans="1:31" x14ac:dyDescent="0.3">
+    <row r="22">
       <c r="A22" s="1">
         <v>1</v>
       </c>
@@ -3173,13 +3038,22 @@
         <v>94</v>
       </c>
       <c r="AD22" s="1">
-        <v>4.7</v>
-      </c>
-      <c r="AE22" s="8" t="s">
+        <v>4.7000000000000002</v>
+      </c>
+      <c r="AE22" t="s">
         <v>189</v>
       </c>
+      <c r="AF22" s="1">
+        <v>4.6459815999999998</v>
+      </c>
+      <c r="AG22" s="1">
+        <v>-74.059867300000008</v>
+      </c>
+      <c r="AH22" t="s">
+        <v>225</v>
+      </c>
     </row>
-    <row r="23" spans="1:31" x14ac:dyDescent="0.3">
+    <row r="23">
       <c r="A23" s="1">
         <v>1</v>
       </c>
@@ -3268,13 +3142,22 @@
         <v>207</v>
       </c>
       <c r="AD23" s="1">
-        <v>4.2</v>
-      </c>
-      <c r="AE23" s="8" t="s">
+        <v>4.2000000000000002</v>
+      </c>
+      <c r="AE23" t="s">
         <v>190</v>
       </c>
+      <c r="AF23" s="1">
+        <v>4.6521540999999997</v>
+      </c>
+      <c r="AG23" s="1">
+        <v>-74.056230099999993</v>
+      </c>
+      <c r="AH23" t="s">
+        <v>226</v>
+      </c>
     </row>
-    <row r="24" spans="1:31" x14ac:dyDescent="0.3">
+    <row r="24">
       <c r="A24" s="1">
         <v>0</v>
       </c>
@@ -3355,13 +3238,22 @@
         <v>11</v>
       </c>
       <c r="AD24" s="1">
-        <v>3.8</v>
-      </c>
-      <c r="AE24" s="8" t="s">
+        <v>3.7999999999999998</v>
+      </c>
+      <c r="AE24" t="s">
         <v>191</v>
       </c>
+      <c r="AF24" s="1">
+        <v>4.7213076999999997</v>
+      </c>
+      <c r="AG24" s="1">
+        <v>-74.040561799999992</v>
+      </c>
+      <c r="AH24" t="s">
+        <v>227</v>
+      </c>
     </row>
-    <row r="25" spans="1:31" x14ac:dyDescent="0.3">
+    <row r="25">
       <c r="A25" s="1">
         <v>1</v>
       </c>
@@ -3450,13 +3342,22 @@
         <v>48</v>
       </c>
       <c r="AD25" s="1">
-        <v>4.2</v>
-      </c>
-      <c r="AE25" s="8" t="s">
+        <v>4.2000000000000002</v>
+      </c>
+      <c r="AE25" t="s">
         <v>192</v>
       </c>
+      <c r="AF25" s="1">
+        <v>4.6764162999999996</v>
+      </c>
+      <c r="AG25" s="1">
+        <v>-74.048835699999998</v>
+      </c>
+      <c r="AH25" t="s">
+        <v>228</v>
+      </c>
     </row>
-    <row r="26" spans="1:31" x14ac:dyDescent="0.3">
+    <row r="26">
       <c r="A26" s="1">
         <v>1</v>
       </c>
@@ -3547,11 +3448,20 @@
       <c r="AD26" s="1">
         <v>4.4000000000000004</v>
       </c>
-      <c r="AE26" s="8" t="s">
+      <c r="AE26" t="s">
         <v>193</v>
       </c>
+      <c r="AF26" s="1">
+        <v>4.6946344</v>
+      </c>
+      <c r="AG26" s="1">
+        <v>-74.032175100000018</v>
+      </c>
+      <c r="AH26" t="s">
+        <v>229</v>
+      </c>
     </row>
-    <row r="27" spans="1:31" x14ac:dyDescent="0.3">
+    <row r="27">
       <c r="A27" s="1">
         <v>1</v>
       </c>
@@ -3642,11 +3552,20 @@
       <c r="AD27" s="1">
         <v>5</v>
       </c>
-      <c r="AE27" s="8" t="s">
+      <c r="AE27" t="s">
         <v>194</v>
       </c>
+      <c r="AF27" s="1">
+        <v>4.6318294999999994</v>
+      </c>
+      <c r="AG27" s="1">
+        <v>-74.072424699999999</v>
+      </c>
+      <c r="AH27" t="s">
+        <v>230</v>
+      </c>
     </row>
-    <row r="28" spans="1:31" x14ac:dyDescent="0.3">
+    <row r="28">
       <c r="A28" s="1">
         <v>1</v>
       </c>
@@ -3733,11 +3652,20 @@
       </c>
       <c r="AC28" s="1"/>
       <c r="AD28" s="1"/>
-      <c r="AE28" s="8" t="s">
-        <v>48</v>
+      <c r="AE28" t="s">
+        <v>48</v>
+      </c>
+      <c r="AF28" s="1">
+        <v>4.6560704</v>
+      </c>
+      <c r="AG28" s="1">
+        <v>-74.054585199999991</v>
+      </c>
+      <c r="AH28" t="s">
+        <v>231</v>
       </c>
     </row>
-    <row r="29" spans="1:31" x14ac:dyDescent="0.3">
+    <row r="29">
       <c r="A29" s="1">
         <v>1</v>
       </c>
@@ -3828,11 +3756,20 @@
       <c r="AD29" s="1">
         <v>4.5</v>
       </c>
-      <c r="AE29" s="8" t="s">
+      <c r="AE29" t="s">
         <v>175</v>
       </c>
+      <c r="AF29" s="1">
+        <v>4.6944631000000001</v>
+      </c>
+      <c r="AG29" s="1">
+        <v>-74.032353299999997</v>
+      </c>
+      <c r="AH29" t="s">
+        <v>232</v>
+      </c>
     </row>
-    <row r="30" spans="1:31" x14ac:dyDescent="0.3">
+    <row r="30">
       <c r="A30" s="1">
         <v>1</v>
       </c>
@@ -3921,13 +3858,22 @@
         <v>518</v>
       </c>
       <c r="AD30" s="1">
-        <v>4.3</v>
-      </c>
-      <c r="AE30" s="8" t="s">
+        <v>4.2999999999999998</v>
+      </c>
+      <c r="AE30" t="s">
         <v>195</v>
       </c>
+      <c r="AF30" s="1">
+        <v>4.6810323999999994</v>
+      </c>
+      <c r="AG30" s="1">
+        <v>-74.046398499999995</v>
+      </c>
+      <c r="AH30" t="s">
+        <v>233</v>
+      </c>
     </row>
-    <row r="31" spans="1:31" x14ac:dyDescent="0.3">
+    <row r="31">
       <c r="A31" s="1">
         <v>1</v>
       </c>
@@ -4007,7 +3953,7 @@
         <v>171</v>
       </c>
       <c r="AA31" s="1">
-        <v>4.2</v>
+        <v>4.2000000000000002</v>
       </c>
       <c r="AB31" s="1">
         <v>1</v>
@@ -4016,13 +3962,22 @@
         <v>334</v>
       </c>
       <c r="AD31" s="1">
-        <v>4.2</v>
-      </c>
-      <c r="AE31" s="8" t="s">
+        <v>4.2000000000000002</v>
+      </c>
+      <c r="AE31" t="s">
         <v>196</v>
       </c>
+      <c r="AF31" s="1">
+        <v>4.6963846</v>
+      </c>
+      <c r="AG31" s="1">
+        <v>-74.044303599999992</v>
+      </c>
+      <c r="AH31" t="s">
+        <v>234</v>
+      </c>
     </row>
-    <row r="32" spans="1:31" x14ac:dyDescent="0.3">
+    <row r="32">
       <c r="A32" s="1">
         <v>1</v>
       </c>
@@ -4111,13 +4066,22 @@
         <v>3</v>
       </c>
       <c r="AD32" s="1">
-        <v>3.3</v>
-      </c>
-      <c r="AE32" s="8" t="s">
+        <v>3.2999999999999998</v>
+      </c>
+      <c r="AE32" t="s">
         <v>197</v>
       </c>
+      <c r="AF32" s="1">
+        <v>4.6674096</v>
+      </c>
+      <c r="AG32" s="1">
+        <v>-74.071941100000004</v>
+      </c>
+      <c r="AH32" t="s">
+        <v>235</v>
+      </c>
     </row>
-    <row r="33" spans="1:31" x14ac:dyDescent="0.3">
+    <row r="33">
       <c r="A33" s="1">
         <v>1</v>
       </c>
@@ -4197,7 +4161,7 @@
         <v>126</v>
       </c>
       <c r="AA33" s="1">
-        <v>3.8</v>
+        <v>3.7999999999999998</v>
       </c>
       <c r="AB33" s="1">
         <v>1</v>
@@ -4206,13 +4170,22 @@
         <v>6</v>
       </c>
       <c r="AD33" s="1">
-        <v>3.7</v>
-      </c>
-      <c r="AE33" s="8" t="s">
+        <v>3.7000000000000002</v>
+      </c>
+      <c r="AE33" t="s">
         <v>198</v>
       </c>
+      <c r="AF33" s="1">
+        <v>4.6130630999999998</v>
+      </c>
+      <c r="AG33" s="1">
+        <v>-74.06663069999999</v>
+      </c>
+      <c r="AH33" t="s">
+        <v>236</v>
+      </c>
     </row>
-    <row r="34" spans="1:31" x14ac:dyDescent="0.3">
+    <row r="34">
       <c r="A34" s="1">
         <v>1</v>
       </c>
@@ -4299,11 +4272,20 @@
       </c>
       <c r="AC34" s="1"/>
       <c r="AD34" s="1"/>
-      <c r="AE34" s="8" t="s">
-        <v>48</v>
+      <c r="AE34" t="s">
+        <v>48</v>
+      </c>
+      <c r="AF34" s="1">
+        <v>4.6521447</v>
+      </c>
+      <c r="AG34" s="1">
+        <v>-74.055869399999992</v>
+      </c>
+      <c r="AH34" t="s">
+        <v>237</v>
       </c>
     </row>
-    <row r="35" spans="1:31" x14ac:dyDescent="0.3">
+    <row r="35">
       <c r="A35" s="1">
         <v>1</v>
       </c>
@@ -4383,7 +4365,7 @@
         <v>87</v>
       </c>
       <c r="AA35" s="1">
-        <v>4.7</v>
+        <v>4.7000000000000002</v>
       </c>
       <c r="AB35" s="1">
         <v>1</v>
@@ -4392,13 +4374,22 @@
         <v>24</v>
       </c>
       <c r="AD35" s="1">
-        <v>4.7</v>
-      </c>
-      <c r="AE35" s="8" t="s">
+        <v>4.7000000000000002</v>
+      </c>
+      <c r="AE35" t="s">
         <v>199</v>
       </c>
+      <c r="AF35" s="1">
+        <v>4.6742881000000001</v>
+      </c>
+      <c r="AG35" s="1">
+        <v>-74.048050799999999</v>
+      </c>
+      <c r="AH35" t="s">
+        <v>238</v>
+      </c>
     </row>
-    <row r="36" spans="1:31" x14ac:dyDescent="0.3">
+    <row r="36">
       <c r="A36" s="1">
         <v>1</v>
       </c>
@@ -4478,18 +4469,27 @@
         <v>85</v>
       </c>
       <c r="AA36" s="1">
-        <v>3.9</v>
+        <v>3.8999999999999999</v>
       </c>
       <c r="AB36" s="1">
         <v>0</v>
       </c>
       <c r="AC36" s="1"/>
       <c r="AD36" s="1"/>
-      <c r="AE36" s="8" t="s">
-        <v>48</v>
+      <c r="AE36" t="s">
+        <v>48</v>
+      </c>
+      <c r="AF36" s="1">
+        <v>4.6009235999999998</v>
+      </c>
+      <c r="AG36" s="1">
+        <v>-74.07176849999999</v>
+      </c>
+      <c r="AH36" t="s">
+        <v>239</v>
       </c>
     </row>
-    <row r="37" spans="1:31" x14ac:dyDescent="0.3">
+    <row r="37">
       <c r="A37" s="1">
         <v>1</v>
       </c>
@@ -4576,11 +4576,20 @@
       </c>
       <c r="AC37" s="1"/>
       <c r="AD37" s="1"/>
-      <c r="AE37" s="8" t="s">
-        <v>48</v>
+      <c r="AE37" t="s">
+        <v>48</v>
+      </c>
+      <c r="AF37" s="1">
+        <v>4.6645292999999999</v>
+      </c>
+      <c r="AG37" s="1">
+        <v>-74.063854599999999</v>
+      </c>
+      <c r="AH37" t="s">
+        <v>240</v>
       </c>
     </row>
-    <row r="38" spans="1:31" x14ac:dyDescent="0.3">
+    <row r="38">
       <c r="A38" s="1">
         <v>1</v>
       </c>
@@ -4671,11 +4680,20 @@
       <c r="AD38" s="1">
         <v>5</v>
       </c>
-      <c r="AE38" s="8" t="s">
+      <c r="AE38" t="s">
         <v>200</v>
       </c>
+      <c r="AF38" s="1">
+        <v>4.6509020999999997</v>
+      </c>
+      <c r="AG38" s="1">
+        <v>-74.057391199999998</v>
+      </c>
+      <c r="AH38" t="s">
+        <v>241</v>
+      </c>
     </row>
-    <row r="39" spans="1:31" x14ac:dyDescent="0.3">
+    <row r="39">
       <c r="A39" s="1">
         <v>1</v>
       </c>
@@ -4764,11 +4782,20 @@
         <v>0</v>
       </c>
       <c r="AD39" s="1"/>
-      <c r="AE39" s="8" t="s">
-        <v>48</v>
+      <c r="AE39" t="s">
+        <v>48</v>
+      </c>
+      <c r="AF39" s="1">
+        <v>4.5965129999999999</v>
+      </c>
+      <c r="AG39" s="1">
+        <v>-74.069208899999992</v>
+      </c>
+      <c r="AH39" t="s">
+        <v>242</v>
       </c>
     </row>
-    <row r="40" spans="1:31" x14ac:dyDescent="0.3">
+    <row r="40">
       <c r="A40" s="1">
         <v>1</v>
       </c>
@@ -4848,18 +4875,27 @@
         <v>11</v>
       </c>
       <c r="AA40" s="1">
-        <v>4.7</v>
+        <v>4.7000000000000002</v>
       </c>
       <c r="AB40" s="1">
         <v>0</v>
       </c>
       <c r="AC40" s="1"/>
       <c r="AD40" s="1"/>
-      <c r="AE40" s="8" t="s">
-        <v>48</v>
+      <c r="AE40" t="s">
+        <v>48</v>
+      </c>
+      <c r="AF40" s="1">
+        <v>4.6574445999999998</v>
+      </c>
+      <c r="AG40" s="1">
+        <v>-74.05652529999999</v>
+      </c>
+      <c r="AH40" t="s">
+        <v>243</v>
       </c>
     </row>
-    <row r="41" spans="1:31" x14ac:dyDescent="0.3">
+    <row r="41">
       <c r="A41" s="1">
         <v>1</v>
       </c>
@@ -4948,13 +4984,22 @@
         <v>1231</v>
       </c>
       <c r="AD41" s="1">
-        <v>4.3</v>
-      </c>
-      <c r="AE41" s="8" t="s">
+        <v>4.2999999999999998</v>
+      </c>
+      <c r="AE41" t="s">
         <v>201</v>
       </c>
+      <c r="AF41" s="1">
+        <v>4.6859608000000001</v>
+      </c>
+      <c r="AG41" s="1">
+        <v>-74.054435400000003</v>
+      </c>
+      <c r="AH41" t="s">
+        <v>244</v>
+      </c>
     </row>
-    <row r="42" spans="1:31" x14ac:dyDescent="0.3">
+    <row r="42">
       <c r="A42" s="1">
         <v>0</v>
       </c>
@@ -5033,11 +5078,19 @@
       </c>
       <c r="AC42" s="1"/>
       <c r="AD42" s="1"/>
-      <c r="AE42" s="8" t="s">
-        <v>48</v>
+      <c r="AE42" t="s">
+        <v>48</v>
+      </c>
+      <c r="AF42" s="1">
+        <v>4.7008947000000001</v>
+      </c>
+      <c r="AG42" s="1">
+        <v>-74.062409000000002</v>
+      </c>
+      <c r="AH42" t="s">
+        <v>245</v>
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>